<commit_message>
feat: refine batch member import flow
</commit_message>
<xml_diff>
--- a/outputs/member-password-template/导出初始密码文件模板.xlsx
+++ b/outputs/member-password-template/导出初始密码文件模板.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始密码" sheetId="1" r:id="R439978a8ac1e4e3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="初始密码" sheetId="1" r:id="Rbf4444b5ebe64b67"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -468,7 +468,7 @@
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="12" t="str">
-        <x:v>示例行仅用于说明文件格式；实际导出时由系统写入本批次成功创建的成员，不包含失败行或已存在账号。</x:v>
+        <x:v>登录账号支持电话或邮箱，单个单元格填写其中一个；示例行仅用于说明格式，实际文件仅包含本批次成功创建的成员。</x:v>
       </x:c>
       <x:c r="B3" s="12"/>
       <x:c r="C3" s="12"/>
@@ -483,7 +483,7 @@
         <x:v>成员名称</x:v>
       </x:c>
       <x:c r="C5" s="22" t="str">
-        <x:v>登录账号</x:v>
+        <x:v>登录账号（电话 / 邮箱）</x:v>
       </x:c>
       <x:c r="D5" s="22" t="str">
         <x:v>归属部门</x:v>

</xml_diff>